<commit_message>
updated from 13 -25
</commit_message>
<xml_diff>
--- a/12621571.xlsx
+++ b/12621571.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\szaid\OneDrive\Desktop\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9A31D662-725C-43A2-86E8-41E9A50D9F69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F16849-8993-4851-8887-45CC7AAFD58B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="612" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="66">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -2675,7 +2675,7 @@
         <v>60</v>
       </c>
       <c r="I38" s="15">
-        <f t="shared" ref="I38:I69" si="2">IF(SUM(B38:F38,H38)=0,"",SUM(B38:F38,H38))</f>
+        <f t="shared" ref="I38:I56" si="2">IF(SUM(B38:F38,H38)=0,"",SUM(B38:F38,H38))</f>
         <v>790</v>
       </c>
       <c r="J38" s="15">
@@ -3175,7 +3175,9 @@
       <c r="M49" s="16" t="s">
         <v>58</v>
       </c>
-      <c r="N49" s="17"/>
+      <c r="N49" s="17" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="50" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="13">
@@ -3222,50 +3224,20 @@
       <c r="N50" s="17"/>
     </row>
     <row r="51" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="13">
-        <v>46291</v>
-      </c>
-      <c r="B51" s="14">
-        <v>540</v>
-      </c>
-      <c r="C51" s="14">
-        <v>90</v>
-      </c>
-      <c r="D51" s="14">
-        <v>50</v>
-      </c>
-      <c r="E51" s="14">
-        <v>30</v>
-      </c>
-      <c r="F51" s="14">
-        <v>0</v>
-      </c>
-      <c r="G51" s="14">
-        <v>0</v>
-      </c>
-      <c r="H51" s="14">
-        <v>60</v>
-      </c>
-      <c r="I51" s="15">
-        <f t="shared" si="2"/>
-        <v>770</v>
-      </c>
-      <c r="J51" s="15">
-        <f t="shared" si="1"/>
-        <v>670</v>
-      </c>
-      <c r="K51" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="L51" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="M51" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="N51" s="17" t="s">
-        <v>65</v>
-      </c>
+      <c r="A51" s="13"/>
+      <c r="B51" s="14"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="14"/>
+      <c r="F51" s="14"/>
+      <c r="G51" s="14"/>
+      <c r="H51" s="14"/>
+      <c r="I51" s="15"/>
+      <c r="J51" s="15"/>
+      <c r="K51" s="16"/>
+      <c r="L51" s="16"/>
+      <c r="M51" s="16"/>
+      <c r="N51" s="17"/>
     </row>
     <row r="52" spans="1:14" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="13"/>
@@ -10443,7 +10415,7 @@
       <c r="G378" s="14"/>
       <c r="H378" s="14"/>
       <c r="I378" s="15" t="str">
-        <f t="shared" ref="I378:I441" si="13">IF(SUM(B378:F378,H378)=0,"",SUM(B378:F378,H378))</f>
+        <f t="shared" ref="I378:I401" si="13">IF(SUM(B378:F378,H378)=0,"",SUM(B378:F378,H378))</f>
         <v/>
       </c>
       <c r="J378" s="15" t="str">
@@ -10711,7 +10683,7 @@
         <v/>
       </c>
       <c r="J390" s="15" t="str">
-        <f t="shared" ref="J390:J453" si="14">IF(I390="","",1440-I390)</f>
+        <f t="shared" ref="J390:J401" si="14">IF(I390="","",1440-I390)</f>
         <v/>
       </c>
       <c r="K390" s="16"/>

</xml_diff>